<commit_message>
Move url generator func to search_utils. All name-to-link conversions mapped
</commit_message>
<xml_diff>
--- a/link_mappings.xlsx
+++ b/link_mappings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\AutoTraderScraper\car_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\AutoTraderScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBE1392-398B-449D-8D97-AC553697DAFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C86DB1D-1BF4-477E-AD2A-87093C4EC10A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38385" yWindow="0" windowWidth="19215" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
+    <workbookView xWindow="14430" yWindow="15" windowWidth="28785" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Create basic Settings page to test input components. Uses index-based values for sliders, which still need mapping
</commit_message>
<xml_diff>
--- a/link_mappings.xlsx
+++ b/link_mappings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\AutoTraderScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C86DB1D-1BF4-477E-AD2A-87093C4EC10A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB3172A-8576-4341-8C16-3DA1D27DB480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14430" yWindow="15" windowWidth="28785" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28785" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -459,12 +459,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -479,10 +485,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -863,22 +870,26 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I2" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="K2" t="s">
@@ -886,42 +897,50 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="I3" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I4" t="s">
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="2" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1466,5 +1485,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add all options values. Improve Settings page layout
</commit_message>
<xml_diff>
--- a/link_mappings.xlsx
+++ b/link_mappings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Coding\AutoTraderScraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB3172A-8576-4341-8C16-3DA1D27DB480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD42147D-9EFC-4253-BF56-D711503BDF7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28785" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
+    <workbookView xWindow="28785" yWindow="0" windowWidth="28815" windowHeight="16200" xr2:uid="{54A614A8-43E4-4466-9419-14EA371F2479}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -296,9 +296,6 @@
     <t>['Include', 'Exclude', 'Show only']</t>
   </si>
   <si>
-    <t>['Four', 'Front', 'Rear'</t>
-  </si>
-  <si>
     <t>['03U', '05U', '10U', '20U', '30U', '40U', '50U']</t>
   </si>
   <si>
@@ -401,9 +398,6 @@
     <t>zero-to-60=4_TO_6</t>
   </si>
   <si>
-    <t>['TO_4', '4_TO_6', '6_TO_8', 8_TO_10', '10_TO_12', 'OVER_12']</t>
-  </si>
-  <si>
     <t>fuel-consumption=OVER_30</t>
   </si>
   <si>
@@ -444,6 +438,12 @@
   </si>
   <si>
     <t>Include = Nothing in link. Exclude = 'exclude-writeoff-categories=on'. Show only = 'only-writeoff-categories=on'. Only 1 of 3 these 3 possible</t>
+  </si>
+  <si>
+    <t>['TO_4', '4_TO_6', '6_TO_8', '8_TO_10', '10_TO_12', 'OVER_12']</t>
+  </si>
+  <si>
+    <t>['Four', 'Front', 'Rear']</t>
   </si>
 </sst>
 </file>
@@ -487,9 +487,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,10 +842,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -870,26 +870,26 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="1" t="s">
         <v>36</v>
       </c>
       <c r="K2" t="s">
@@ -897,68 +897,68 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>97</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>98</v>
-      </c>
       <c r="C5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>62</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I5" t="s">
         <v>63</v>
@@ -968,16 +968,16 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" t="s">
         <v>99</v>
       </c>
-      <c r="C6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>73</v>
       </c>
       <c r="I6" t="s">
@@ -992,12 +992,12 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>57</v>
       </c>
       <c r="I7" t="s">
@@ -1012,12 +1012,12 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
-      </c>
-      <c r="E8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>58</v>
       </c>
       <c r="I8" t="s">
@@ -1028,16 +1028,16 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>54</v>
       </c>
       <c r="I9" t="s">
@@ -1048,16 +1048,16 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
-      </c>
-      <c r="E10" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>54</v>
       </c>
       <c r="I10" t="s">
@@ -1072,16 +1072,16 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" t="s">
         <v>107</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" t="s">
         <v>108</v>
-      </c>
-      <c r="E11" t="s">
-        <v>74</v>
-      </c>
-      <c r="G11" t="s">
-        <v>109</v>
       </c>
       <c r="I11" t="s">
         <v>53</v>
@@ -1095,16 +1095,16 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I12" t="s">
         <v>52</v>
@@ -1118,16 +1118,16 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
-      </c>
-      <c r="E13" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>41</v>
       </c>
       <c r="G13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I13" t="s">
         <v>51</v>
@@ -1141,16 +1141,16 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" t="s">
         <v>112</v>
-      </c>
-      <c r="C14" t="s">
-        <v>108</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
-      <c r="G14" t="s">
-        <v>113</v>
       </c>
       <c r="I14" t="s">
         <v>50</v>
@@ -1164,16 +1164,16 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
-      </c>
-      <c r="E15" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>75</v>
       </c>
       <c r="G15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I15" t="s">
         <v>49</v>
@@ -1187,16 +1187,16 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
-      </c>
-      <c r="E16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>76</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I16" t="s">
         <v>48</v>
@@ -1210,12 +1210,12 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>100</v>
-      </c>
-      <c r="E17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>77</v>
       </c>
       <c r="I17" t="s">
@@ -1230,12 +1230,12 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
-      </c>
-      <c r="E18" t="s">
+        <v>99</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>77</v>
       </c>
       <c r="I18" t="s">
@@ -1250,12 +1250,12 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>43</v>
       </c>
       <c r="I19" t="s">
@@ -1270,12 +1270,12 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" t="s">
+        <v>99</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>43</v>
       </c>
       <c r="I20" t="s">
@@ -1290,16 +1290,16 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C21" t="s">
-        <v>108</v>
-      </c>
-      <c r="E21" t="s">
-        <v>121</v>
+        <v>107</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>134</v>
       </c>
       <c r="G21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I21" t="s">
         <v>67</v>
@@ -1313,13 +1313,13 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
-      </c>
-      <c r="E22" t="s">
-        <v>91</v>
+        <v>99</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="I22" t="s">
         <v>84</v>
@@ -1333,13 +1333,13 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
-      </c>
-      <c r="E23" t="s">
-        <v>90</v>
+        <v>99</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="I23" t="s">
         <v>68</v>
@@ -1353,13 +1353,13 @@
         <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
-      </c>
-      <c r="E24" t="s">
-        <v>89</v>
+        <v>99</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="I24" t="s">
         <v>82</v>
@@ -1373,16 +1373,16 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
-      </c>
-      <c r="E25" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G25" t="s">
         <v>87</v>
-      </c>
-      <c r="G25" t="s">
-        <v>88</v>
       </c>
       <c r="I25" t="s">
         <v>83</v>
@@ -1396,16 +1396,16 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
-      </c>
-      <c r="E26" t="s">
-        <v>86</v>
+        <v>107</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="G26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I26" t="s">
         <v>69</v>
@@ -1419,16 +1419,16 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
+        <v>125</v>
+      </c>
+      <c r="C27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C27" t="s">
-        <v>108</v>
-      </c>
-      <c r="E27" t="s">
-        <v>129</v>
-      </c>
       <c r="G27" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="I27" t="s">
         <v>70</v>
@@ -1442,16 +1442,16 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
-      </c>
-      <c r="E28" t="s">
-        <v>131</v>
+        <v>107</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="G28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I28" t="s">
         <v>71</v>
@@ -1465,22 +1465,22 @@
         <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C29" t="s">
+        <v>131</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G29" t="s">
         <v>133</v>
-      </c>
-      <c r="E29" t="s">
-        <v>85</v>
-      </c>
-      <c r="G29" t="s">
-        <v>135</v>
       </c>
       <c r="I29" t="s">
         <v>72</v>
       </c>
       <c r="J29" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>